<commit_message>
feat(analytics): add Word report (.docx) generation with strict formatting
</commit_message>
<xml_diff>
--- a/data/output/top_municipalities.xlsx
+++ b/data/output/top_municipalities.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t>Место</t>
   </si>
@@ -32,65 +32,69 @@
     <t>Омск г.о.</t>
   </si>
   <si>
-    <t>Одесский район</t>
-  </si>
-  <si>
-    <t>Черлакский район</t>
-  </si>
-  <si>
-    <t>Уборка дорог от снега и наледи, Изменение класса и количества подвижного состава на маршрутах общественного транспорта, Содержание и ремонт образовательных организаций</t>
-  </si>
-  <si>
-    <t>Отсутствие холодной и/или горячей воды</t>
-  </si>
-  <si>
-    <t>Ненадлежащее качество или отключение отопления</t>
-  </si>
-  <si>
-    <t>Исилькульский район</t>
+    <t>Омская область, другое</t>
   </si>
   <si>
     <t>Тарский район</t>
   </si>
   <si>
-    <t>Омская область, другое</t>
-  </si>
-  <si>
-    <t>Тевризский район</t>
-  </si>
-  <si>
-    <t>Называевский район</t>
-  </si>
-  <si>
-    <t>Уборка дорог от снега и наледи, Изменение класса и количества подвижного состава на маршрутах общественного транспорта, Оказание платных медицинских услуг</t>
-  </si>
-  <si>
-    <t>Уборка дорог от снега и наледи</t>
-  </si>
-  <si>
-    <t>Единое пособие на детей (задержка выплаты, отказ, оформление)</t>
-  </si>
-  <si>
-    <t>Спортивные мероприятия</t>
-  </si>
-  <si>
-    <t>Плата за жилое помещение, предоставление коммунальных и иных услуг (ЖКУ)</t>
+    <t>Уборка дорог от снега и наледи, Ненадлежащее качество или отключение отопления, Аварии (в т.ч. прорывы) в системе водоснабжения</t>
+  </si>
+  <si>
+    <t>Единое пособие на детей (задержка выплаты, отказ, оформление), Поддержка сирот (запрос помощи, предоставление жилья, отказ и т.д.), Поддержка иных категорий граждан (запрос помощи, задержка выплат, отказ и т.д.)</t>
+  </si>
+  <si>
+    <t>Уборка дорог от снега и наледи, Отсутствие холодной и/или горячей воды, Ненадлежащее качество или отключение отопления</t>
+  </si>
+  <si>
+    <t>Омский район</t>
+  </si>
+  <si>
+    <t>Муромцевский район</t>
+  </si>
+  <si>
+    <t>Калачинский район</t>
+  </si>
+  <si>
+    <t>Большереченский район</t>
+  </si>
+  <si>
+    <t>Любинский район</t>
+  </si>
+  <si>
+    <t>Москаленский район</t>
+  </si>
+  <si>
+    <t>Азовский немецкий национальный район</t>
+  </si>
+  <si>
+    <t>Изменение, отмена или добавление маршрутов общественного транспорта, Ненадлежащее качество или отключение отопления, Отсутствие холодной и/или горячей воды</t>
+  </si>
+  <si>
+    <t>Отсутствие холодной и/или горячей воды, Уборка дорог от снега и наледи, Ненадлежащее качество или отключение отопления</t>
+  </si>
+  <si>
+    <t>Плохое качество воды, Уборка дорог от снега и наледи, График движения общественного транспорта</t>
+  </si>
+  <si>
+    <t>Ненадлежащее качество или отключение отопления, Отсутствие холодной и/или горячей воды, Уборка дорог от снега и наледи</t>
+  </si>
+  <si>
+    <t>Водоразборные колонки, колодцы, Нарушение при обращении с отходами (слив ЖБО, сброс мусора и др.), Отсутствие холодной и/или горячей воды</t>
+  </si>
+  <si>
+    <t>Уборка дорог от снега и наледи, Эпидемии и болезни сельскохозяйственных животных, Проблемы с отоплением в социальных учреждениях</t>
+  </si>
+  <si>
+    <t>Содержание и ремонт образовательных организаций, График движения общественного транспорта, Подтопление территории (кроме дорог) из-за дождей, работа и ремонт ливневых канализаций</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -106,7 +110,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -114,30 +118,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,16 +422,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -457,7 +443,7 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>43042</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -471,7 +457,7 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>1523</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -485,7 +471,7 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>1430</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -498,20 +484,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -523,10 +509,10 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>43042</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -534,13 +520,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>1523</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -548,13 +534,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>1430</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -565,10 +551,10 @@
         <v>10</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>1389</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -579,10 +565,10 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>1106</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -593,10 +579,10 @@
         <v>12</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>1101</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -607,10 +593,10 @@
         <v>13</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1015</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -621,10 +607,38 @@
         <v>14</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>374</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10">
+        <v>277</v>
+      </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>268</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>